<commit_message>
Update zipper bag cost workbook
</commit_message>
<xml_diff>
--- a/Zipper bag/报价计算方式.xlsx
+++ b/Zipper bag/报价计算方式.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Ai项目\世科报价系统\Zipper bag\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFA5235A-3003-4773-82DF-D7BC8FF56996}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C09A5E7-9DB6-4210-B11D-F5A6EAA5E47E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="55">
   <si>
     <t>长（mm)</t>
     <phoneticPr fontId="3" type="noConversion"/>
@@ -131,10 +131,6 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>袋本体原料成本</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>水墨成本</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -234,12 +230,6 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>报价时粗略估计，
-夹链部分重量占10%，
-袋本体占90%。</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>夹链混合原料成本</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -249,6 +239,19 @@
   </si>
   <si>
     <t>注意：袋子重量不是外界输入，而是需要系统根据前边输入的产品规格计算出来</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>该值由用户输入，
+默认值10%</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>袋本体原料成本（不含夹链）</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>夹链原料成本</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -320,7 +323,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -442,6 +445,32 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
@@ -451,7 +480,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -500,6 +529,27 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -522,28 +572,16 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -813,10 +851,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AA583AD-8CB7-4F0C-A681-D6779EC3025D}">
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.6640625" customWidth="1"/>
+    <col min="1" max="1" width="26.19921875" customWidth="1"/>
     <col min="2" max="2" width="14.265625" customWidth="1"/>
     <col min="3" max="3" width="38.1328125" customWidth="1"/>
     <col min="4" max="4" width="18.6640625" customWidth="1"/>
@@ -826,26 +864,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="25"/>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
+      <c r="A2" s="17"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
     </row>
     <row r="3" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="24" t="s">
+      <c r="A3" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="24"/>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
+      <c r="B3" s="16"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
     </row>
     <row r="4" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
@@ -883,16 +921,16 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>45</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>46</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
@@ -924,14 +962,14 @@
       </c>
     </row>
     <row r="9" spans="1:7" ht="20.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="26" t="s">
+      <c r="A9" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="27"/>
-      <c r="C9" s="27"/>
-      <c r="D9" s="28"/>
+      <c r="B9" s="19"/>
+      <c r="C9" s="19"/>
+      <c r="D9" s="20"/>
       <c r="E9" s="11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.3">
@@ -942,32 +980,31 @@
       <c r="C10" s="13">
         <v>0.7</v>
       </c>
-      <c r="D10" s="21">
+      <c r="D10" s="28">
+        <f>1-D13</f>
         <v>0.9</v>
       </c>
-      <c r="E10" s="15" t="s">
-        <v>50</v>
-      </c>
+      <c r="E10" s="32"/>
     </row>
     <row r="11" spans="1:7" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="20" t="s">
+      <c r="A11" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="20"/>
+      <c r="B11" s="27"/>
       <c r="C11" s="13">
         <v>0.3</v>
       </c>
-      <c r="D11" s="21"/>
-      <c r="E11" s="23"/>
+      <c r="D11" s="28"/>
+      <c r="E11" s="33"/>
     </row>
     <row r="12" spans="1:7" ht="21.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="16" t="s">
-        <v>48</v>
-      </c>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="16"/>
-      <c r="E12" s="23"/>
+      <c r="A12" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="B12" s="23"/>
+      <c r="C12" s="23"/>
+      <c r="D12" s="23"/>
+      <c r="E12" s="30"/>
     </row>
     <row r="13" spans="1:7" ht="18.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="15" t="s">
@@ -977,10 +1014,12 @@
       <c r="C13" s="12">
         <v>0.02</v>
       </c>
-      <c r="D13" s="22">
+      <c r="D13" s="29">
         <v>0.1</v>
       </c>
-      <c r="E13" s="23"/>
+      <c r="E13" s="32" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="15" t="s">
@@ -991,15 +1030,15 @@
         <v>0.98</v>
       </c>
       <c r="D14" s="15"/>
-      <c r="E14" s="23"/>
+      <c r="E14" s="31"/>
       <c r="F14" s="9"/>
     </row>
     <row r="15" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="29" t="s">
+      <c r="A15" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="24"/>
-      <c r="C15" s="30"/>
+      <c r="B15" s="16"/>
+      <c r="C15" s="22"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
@@ -1047,7 +1086,7 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B20" s="4">
         <v>300</v>
@@ -1090,15 +1129,15 @@
       </c>
     </row>
     <row r="25" spans="1:3" ht="17.649999999999999" x14ac:dyDescent="0.3">
-      <c r="A25" s="17" t="s">
-        <v>26</v>
-      </c>
-      <c r="B25" s="18"/>
-      <c r="C25" s="19"/>
+      <c r="A25" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="B25" s="25"/>
+      <c r="C25" s="26"/>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B26" s="4">
         <f>(B16*C10+B17*C11)</f>
@@ -1110,7 +1149,7 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B27" s="4">
         <f>B16*C14+B18*C13</f>
@@ -1122,94 +1161,109 @@
     </row>
     <row r="28" spans="1:3" ht="27" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B28" s="4">
         <v>11.5</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="21.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B29" s="5">
+        <f>B28*D10*B26/1000000</f>
+        <v>0.13041</v>
+      </c>
+      <c r="C29" s="5"/>
+    </row>
+    <row r="30" spans="1:3" ht="21.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B30" s="5">
+        <f>B28*D13*B27/1000000</f>
+        <v>1.5674500000000001E-2</v>
+      </c>
+      <c r="C30" s="5"/>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B29" s="5">
-        <f>B28*0.9*B26/1000000+B28*0.1*B27/1000000</f>
-        <v>0.14608450000000001</v>
-      </c>
-      <c r="C29" s="5"/>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B30" s="5">
+      <c r="B31" s="5">
         <f>IF(B8="否",0,IF(B8="一色",18*B19/D8,IF(B8="二色",18*B19/D8*2,"")))</f>
         <v>3.2399999999999998E-3</v>
       </c>
-      <c r="C30" s="6" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A31" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B31" s="5">
+      <c r="C31" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B32" s="5">
         <f>IF(B8="否",0,IF(B8="一色",300/(100000/D4*1000),IF(B8="二色",300/(100000/D4*1000)*2,"")))</f>
         <v>8.0999999999999996E-4</v>
       </c>
-      <c r="C31" s="6" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A32" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B32" s="5">
+      <c r="C32" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B33" s="5">
         <f>0.7*B22/1000/B7</f>
         <v>5.3666666666666652E-4</v>
       </c>
-      <c r="C32" s="6" t="s">
+      <c r="C33" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" s="1" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A33" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B33" s="5">
+      <c r="B34" s="5">
         <f>B21/B7</f>
         <v>1.3666666666666666E-2</v>
       </c>
-      <c r="C33" s="5"/>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A34" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B34" s="5">
+      <c r="C34" s="5"/>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B35" s="5">
         <f>B23/B7/D7</f>
         <v>4.3055555555555555E-3</v>
       </c>
-      <c r="C34" s="5"/>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A35" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B35" s="5">
-        <f>SUM(B29:B34)</f>
+      <c r="C35" s="5"/>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B36" s="5">
+        <f>SUM(B29:B35)</f>
         <v>0.16864338888888888</v>
       </c>
-      <c r="C35" s="5"/>
+      <c r="C36" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="13">
-    <mergeCell ref="E10:E14"/>
+  <mergeCells count="14">
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="D10:D11"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="E10:E11"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="A1:D2"/>
     <mergeCell ref="A9:D9"/>
@@ -1218,10 +1272,6 @@
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="A14:B14"/>
     <mergeCell ref="A12:D12"/>
-    <mergeCell ref="A25:C25"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="D10:D11"/>
-    <mergeCell ref="D13:D14"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <dataValidations count="4">
@@ -1249,37 +1299,37 @@
   <sheetData>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B2" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="C2" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="C2" s="11" t="s">
-        <v>40</v>
-      </c>
       <c r="D2" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E2" s="11" t="s">
         <v>15</v>
       </c>
       <c r="F2" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="G2" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="H2" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="I2" s="11" t="s">
         <v>43</v>
-      </c>
-      <c r="G2" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="H2" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="I2" s="11" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B3">
         <f>原材料成本计算方法!B29</f>
-        <v>0.14608450000000001</v>
+        <v>0.13041</v>
       </c>
       <c r="C3" t="e">
         <f>原材料成本计算方法!#REF!</f>
@@ -1290,19 +1340,19 @@
         <v>#REF!</v>
       </c>
       <c r="E3">
-        <f>原材料成本计算方法!B30+原材料成本计算方法!B31</f>
+        <f>原材料成本计算方法!B31+原材料成本计算方法!B32</f>
         <v>4.0499999999999998E-3</v>
       </c>
       <c r="F3">
-        <f>原材料成本计算方法!B32</f>
+        <f>原材料成本计算方法!B33</f>
         <v>5.3666666666666652E-4</v>
       </c>
       <c r="G3">
-        <f>原材料成本计算方法!B33</f>
+        <f>原材料成本计算方法!B34</f>
         <v>1.3666666666666666E-2</v>
       </c>
       <c r="H3">
-        <f>原材料成本计算方法!B34</f>
+        <f>原材料成本计算方法!B35</f>
         <v>4.3055555555555555E-3</v>
       </c>
       <c r="I3" t="e">

</xml_diff>